<commit_message>
Módulo 3: quita los retos finales (hoja Consigna, proyecto integrador y lista de entrega)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Modulo3-Base-Servicios.xlsx
+++ b/Modulo3-Base-Servicios.xlsx
@@ -5,7 +5,6 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="Servicios" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Consigna" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
@@ -9990,124 +9989,4 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:B22"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="100" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B2" s="3" t="s">
-        <v>391</v>
-      </c>
-    </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B3" s="4" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B5" s="5" t="s">
-        <v>394</v>
-      </c>
-    </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B6" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B7" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B8" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B11" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B12" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B13" s="5" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B14" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B15" s="5" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B16" s="6" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" s="6" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="6" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19" s="6" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B20" s="6" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B22" s="4" t="s">
-        <v>408</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
 </file>
</xml_diff>